<commit_message>
feat(wechat): enhance WeChat bill importer to parse payee names and support new transaction types
</commit_message>
<xml_diff>
--- a/examples/import_only/documents/Assets/Payment/Wechat/2019-09-30.微信支付账单流水文件(20190801-20190930)——【解压密码可在微信支付公众号查看】.xlsx
+++ b/examples/import_only/documents/Assets/Payment/Wechat/2019-09-30.微信支付账单流水文件(20190801-20190930)——【解压密码可在微信支付公众号查看】.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aqnin\Projects\beancount-daoru\examples\import_only\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9D659A-CF27-4976-89BC-2FA8481EE965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14206C2-41F6-479A-AD3C-425DF587F0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="170">
   <si>
     <t>微信支付账单明细</t>
   </si>
@@ -521,6 +521,17 @@
   </si>
   <si>
     <t>4. 本账单中所有时间均为UTC+08:00时间</t>
+  </si>
+  <si>
+    <t>微信红包（单发）</t>
+  </si>
+  <si>
+    <t>发给张三</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">156823045120240607AQEQJ8ZY4Q	</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1513,7 +1524,7 @@
         <v>34</v>
       </c>
       <c r="F28" s="1">
-        <v>548.58</v>
+        <v>548.58000000000004</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>56</v>
@@ -1863,7 +1874,7 @@
         <v>38</v>
       </c>
       <c r="F38" s="1">
-        <v>0.07</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>34</v>
@@ -1898,7 +1909,7 @@
         <v>38</v>
       </c>
       <c r="F39" s="1">
-        <v>0.07</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>34</v>
@@ -2263,16 +2274,39 @@
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A50" s="2"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
-      <c r="I50" s="3"/>
-      <c r="J50" s="3"/>
-      <c r="K50" s="3"/>
+      <c r="A50" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F50" s="1">
+        <v>100</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A51" s="2"/>
@@ -2757,6 +2791,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A7:K7"/>
+    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="A10:K10"/>
     <mergeCell ref="A17:K17"/>
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="A12:K12"/>
@@ -2764,16 +2808,6 @@
     <mergeCell ref="A14:K14"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="A7:K7"/>
-    <mergeCell ref="A8:K8"/>
-    <mergeCell ref="A9:K9"/>
-    <mergeCell ref="A10:K10"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>